<commit_message>
Add INV+PKL pairing (BHC-first) and require HS on MA/PT lines.
GUI shows a rematchable pairing table under Selected files; split PKL
supplies packages/GW while format_id stays on INV/combined. hard_check
now conflicts if any MA/PT line item lacks hs_code (BHC unchanged).
</commit_message>
<xml_diff>
--- a/data/templates/InvoiceExtract_Template.xlsx
+++ b/data/templates/InvoiceExtract_Template.xlsx
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -685,10 +685,35 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>inv_file</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>pkl_file</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>pkl_used</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>pair_status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>error</t>
         </is>

</xml_diff>

<commit_message>
Add Summary BL columns + BHC arrival/HBL formats (cases 2–6).
Wire BL No./Packages/G.W. into Result Summary (no overwrite of invoice
pkg/GW), pair 提單 in GUI, and seed ceva/dhl/hippopo layout families.
</commit_message>
<xml_diff>
--- a/data/templates/InvoiceExtract_Template.xlsx
+++ b/data/templates/InvoiceExtract_Template.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -482,25 +482,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>BL No.</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BL Packages</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BL G.W. (kgs)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Incoterms</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Invoice Value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>LINE</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Invoice Currency</t>
         </is>
@@ -603,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -705,15 +720,30 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>bl_file</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>bl_used</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>bl_format_id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>pair_status</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>error</t>
         </is>

</xml_diff>

<commit_message>
Move Summary BL columns to far right; unify header style; brand GUI.
Reorder BL No./Packages/G.W. after Invoice Currency in template and
export write path, apply one shared Summary header fill/font/alignment
(including when rewriting headers), and show Published by Peter Yang on
the Tk window title and footer. Add review screenshots and tests.
</commit_message>
<xml_diff>
--- a/data/templates/InvoiceExtract_Template.xlsx
+++ b/data/templates/InvoiceExtract_Template.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -49,7 +54,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -71,13 +76,22 @@
         <color rgb="00B4B4B4"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -457,67 +471,70 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Invoice No.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Packages</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Package Mode</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>G.W. (kgs)-Air DIM. (CBM)-Sea</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Incoterms</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Value</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>LINE</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Invoice Currency</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>BL No.</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>BL Packages</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>BL G.W. (kgs)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Incoterms</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Invoice Value</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>LINE</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Invoice Currency</t>
         </is>
       </c>
     </row>
@@ -550,57 +567,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Des</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Unt</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Amt</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>UoM</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Co</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>HS code</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>N.W.</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>InvoiceNumber</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
@@ -638,112 +655,112 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>format_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>text_backend</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>checker_verdict</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>needs_gold</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>needs_ocr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>labeled_amount</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>labeled_amount_label</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>checker_issues</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>checker_details</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>inv_file</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>pkl_file</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>pkl_used</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>bl_file</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>bl_used</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>bl_format_id</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>pair_status</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>error</t>
         </is>

</xml_diff>

<commit_message>
Color Summary BL headers green.
</commit_message>
<xml_diff>
--- a/data/templates/InvoiceExtract_Template.xlsx
+++ b/data/templates/InvoiceExtract_Template.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00008000"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,12 +91,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -522,17 +530,17 @@
           <t>Invoice Currency</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>BL No.</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>BL Packages</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>BL G.W. (kgs)</t>
         </is>

</xml_diff>

<commit_message>
Ensure Excel exports use Calibri consistently
Apply Calibri to headers and every written cell while preserving existing header styling, and update the bundled template with regression coverage.
</commit_message>
<xml_diff>
--- a/data/templates/InvoiceExtract_Template.xlsx
+++ b/data/templates/InvoiceExtract_Template.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
@@ -91,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -100,6 +106,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,62 +497,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Invoice No.</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Packages</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Package Mode</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>G.W. (kgs)-Air DIM. (CBM)-Sea</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Incoterms</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Invoice Value</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>LINE</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Invoice Currency</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>BL No.</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>BL Packages</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>BL G.W. (kgs)</t>
         </is>
@@ -575,57 +587,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>PN</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Des</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Unt</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Amt</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>UoM</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Co</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>HS code</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>N.W.</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>InvoiceNumber</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
@@ -663,112 +675,112 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>format_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>text_backend</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>checker_verdict</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>needs_gold</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>needs_ocr</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>labeled_amount</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>labeled_amount_label</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>checker_issues</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>checker_details</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>inv_file</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>pkl_file</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>pkl_used</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>bl_file</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>bl_used</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>bl_format_id</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>pair_status</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>error</t>
         </is>

</xml_diff>